<commit_message>
docs: apply owner decisions to document templates (B2B forms, numbering PM2026-NNNNN, xlsx layout, NDS/date rules) + track source docx; fix .gitignore encoding
</commit_message>
<xml_diff>
--- a/templates_result/01_variables_register.xlsx
+++ b/templates_result/01_variables_register.xlsx
@@ -447,8 +447,6 @@
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="45" customWidth="1" min="8" max="8"/>
     <col width="62" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1"/>
@@ -549,7 +547,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>⚠ уточнить схему нумерации (см. № 64, 65)</t>
+          <t>единый номер пакета: договор = проект `ПМ2026-NNNNN` (05-В1)</t>
         </is>
       </c>
     </row>
@@ -640,9 +638,9 @@
           <t>текст</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>*только если заказаны сборка/монтаж (`Order.hasAssembly`)</t>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>*только если заказаны сборка/монтаж (`Order.hasAssembly`); № = единый номер пакета (05-В2)</t>
         </is>
       </c>
     </row>
@@ -731,12 +729,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>текст, суффикс «ПМ-26» в оригинале</t>
+          <t>текст «ПМ2026-NNNNN»</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>⚠ уточнить схему «№ ___ ПМ-26» (см. 05-В)</t>
+          <t>единый номер пакета (05-В1); хвост «ПМ-26» в шапках не печатается</t>
         </is>
       </c>
     </row>
@@ -778,12 +776,12 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>текст «№ ___ ПМ-26»</t>
+          <t>текст «ПМ2026-NNNNN»</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>может совпадать с № 5 — ⚠ уточнить</t>
+          <t>совпадает с № 5 — единый номер пакета (05-В2)</t>
         </is>
       </c>
     </row>
@@ -830,7 +828,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>*только при заказе монтажа</t>
+          <t>*только при заказе монтажа; № по умолчанию = единый номер пакета (05-В2)</t>
         </is>
       </c>
     </row>
@@ -850,9 +848,9 @@
           <t>Дата подписания Акта приёма-передачи Товара (= дата передачи товара)</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>АПП: шапка и подписи; ГТ T1 «Дата передачи Товара»; ПРАВ: титульная дата (⚠)</t>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>АПП: шапка и подписи; ГТ T1 «Дата передачи Товара»; ПРАВ: титульная дата (= дата выдачи при передаче, 05-Ж2)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -969,7 +967,11 @@
           <t>текст</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>по умолчанию = единый номер пакета (05-В2)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1041,7 +1043,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>⚠ дата выдачи при передаче товара или дата ДКП</t>
+          <t>Проект: дата передачи товара</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1061,7 +1063,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>⚠ уточнить, какая дата ставится</t>
+          <t>дата выдачи при передаче Товара = `Doc.actAcceptance.date` (05-Ж2)</t>
         </is>
       </c>
     </row>
@@ -1209,7 +1211,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>⚠ в ТЗ контакт физлица: «фио, телефон, адрес» — разбивка на поля ⚠ уточнить</t>
+          <t>разбивка на поля подтверждена (05-А1)</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1285,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Карточка клиента</t>
+          <t>Расчётное: ФИО (отчество)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1303,7 +1305,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>⚠ в ТЗ не описано; вариант: вычислять по отчеству либо добавить поле</t>
+          <t>вычисляется по отчеству (‑вич/‑вна), иначе по имени (05-А2)</t>
         </is>
       </c>
     </row>
@@ -1350,7 +1352,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>⚠ поля в CRM не описаны в ТЗ — добавить</t>
+          <t>есть в CRM (05-А1)</t>
         </is>
       </c>
     </row>
@@ -1397,7 +1399,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>⚠ добавить</t>
+          <t>есть в CRM (05-А1)</t>
         </is>
       </c>
     </row>
@@ -1444,7 +1446,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>⚠ добавить</t>
+          <t>есть в CRM (05-А1)</t>
         </is>
       </c>
     </row>
@@ -1491,7 +1493,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>⚠ добавить</t>
+          <t>есть в CRM (05-А1)</t>
         </is>
       </c>
     </row>
@@ -1538,7 +1540,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>⚠ добавить</t>
+          <t>есть в CRM (05-А1)</t>
         </is>
       </c>
     </row>
@@ -1632,7 +1634,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>для ЮЛ — телефон представителя</t>
+          <t>один общий телефон карточки (для ФЛ и ЮЛ) (05-А4)</t>
         </is>
       </c>
     </row>
@@ -1679,7 +1681,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>в ТЗ контакт = «фио, телефон, адрес» — ⚠ поле email добавить</t>
+          <t>поле добавлено; если пусто — в документ ничего не вносится (05-А3)</t>
         </is>
       </c>
     </row>
@@ -2503,7 +2505,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Проект: номер `ПМ000001` / `ПМ2026-000001` (из ТЗ)</t>
+          <t>Проект: номер `ПМ2026-NNNNN` (единый с договором, 05-В1)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2521,11 +2523,7 @@
           <t>текст</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>см. № 64, 65</t>
-        </is>
-      </c>
+      <c r="I49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3307,7 +3305,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>БЗ: таблица «ПЕРЕЧЕНЬ ИЗДЕЛИЙ» (строки 19–26, макс. 8)</t>
+          <t>БЗ: таблица «ПЕРЕЧЕНЬ ИЗДЕЛИЙ» (строки 19–26, в макете 8 строк)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3332,7 +3330,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>⚠ макет бланка: 8 готовых строк — при большем числе нужна перевёрстка</t>
+          <t>при &gt;8 позициях — вставка строк допустима (05-Е5)</t>
         </is>
       </c>
     </row>
@@ -3377,9 +3375,9 @@
           <t>цикл</t>
         </is>
       </c>
-      <c r="I69" s="3" t="inlineStr">
-        <is>
-          <t>⚠ в макете блок свёрстан вертикально-объединёнными ячейками на 1 позицию — см. 02/СП и 05-Е</t>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>перевёрстка «одна позиция = одна строка» подтверждена (05-Е2)</t>
         </is>
       </c>
     </row>
@@ -3549,7 +3547,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>БЗ: ячейка суммы «ИТОГО» (⚠ точная ячейка не определена); СП</t>
+          <t>БЗ: ячейка G29 (05-Е1); СП</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3574,7 +3572,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>⚠ БЗ: уточнить ячейку суммы ИТОГО (05-Е)</t>
+          <t>БЗ — ячейка G29 (05-Е1)</t>
         </is>
       </c>
     </row>
@@ -3643,7 +3641,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>СП «ИТОГО» (E28), «Со скидкой» (E29)</t>
+          <t>СП: «ИТОГО» (E28), сумма — F28 (05-Е3)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3666,7 +3664,11 @@
           <t>число, руб.</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr"/>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>сумма ИТОГО — F28 (05-Е3)</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3691,7 +3693,7 @@
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>Сделка: сумма КП/скидка (в ТЗ: «сумма планируемая на основании КП»; дизайнерский бонус 10 %)</t>
+          <t>Сделка: сумма КП/скидка (наценка дизайнера 10 % — внутренняя, в документы не выводится, 05-З2)</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3711,7 +3713,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>⚠ уточнить правила скидок/бонуса дизайнера</t>
+          <t>в документы выводится только реальная скидка клиенту (05-З2)</t>
         </is>
       </c>
     </row>
@@ -3758,7 +3760,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>при отсутствии скидки = № 63</t>
+          <t>при отсутствии скидки = № 63; сумма «Со скидкой» — F29 (05-Е3)</t>
         </is>
       </c>
     </row>
@@ -3940,9 +3942,9 @@
           <t>условный текст</t>
         </is>
       </c>
-      <c r="I82" t="inlineStr">
-        <is>
-          <t>в оригинале обе фразы + «(нужное указать)»</t>
+      <c r="I82" s="3" t="inlineStr">
+        <is>
+          <t>по умолчанию «НДС не облагается» (УСН «доходы-расходы», 05-З1); признак — в настройках продавца</t>
         </is>
       </c>
     </row>
@@ -4589,7 +4591,7 @@
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>в оригинальных датах год проставлен «2026» — брать из года генерации, ⚠ уточнить (05-Ж)</t>
+          <t>в оригинальных датах год проставлен «2026» — при генерации брать год проекта (05-Ж1)</t>
         </is>
       </c>
     </row>
@@ -4643,7 +4645,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>печатается пустым «____» — подписывается вручную; при УКЭП — заменяется (⚠)</t>
+          <t>печатается пустым — подпись вручную или по ЭДО (05-Б4)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: close owner questions (addresses 05-D1, no showroom defects list, add survey form & power-of-attorney templates to plan)
</commit_message>
<xml_diff>
--- a/templates_result/01_variables_register.xlsx
+++ b/templates_result/01_variables_register.xlsx
@@ -1585,9 +1585,9 @@
           <t>текст</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>⚠ в ТЗ один «адрес» — нужен ли отдельно адрес регистрации и доставки (см. 05-Д)</t>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>подтверждено (05-Д1): в реквизитах — адрес регистрации; адрес монтажа/доставки — отдельное поле № 43</t>
         </is>
       </c>
     </row>
@@ -2654,7 +2654,7 @@
       </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>⚠ возможно отличается от `Client.regAddress`/юр. адреса — уточнить структуру (05-Д)</t>
+          <t>подтверждено (05-Д1): адрес монтажа/доставки обязателен в тексте договоров (ДМ, АВР, ГТ, БЗ, СП) — отдельное поле</t>
         </is>
       </c>
     </row>

</xml_diff>